<commit_message>
Labeling Part10 Batch A Manual Annotation
</commit_message>
<xml_diff>
--- a/03_Labeling/outputs/full_annotation/full_annotation_381.xlsx
+++ b/03_Labeling/outputs/full_annotation/full_annotation_381.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Penelitian Sentimen Bencana Nasional\03_Labeling\outputs\full_annotation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D0EEC4A-7C39-4048-B6FA-65C63BCC2496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FFB09E0-5C95-49DF-8E06-D822E1E46F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4737" uniqueCount="2188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4745" uniqueCount="2190">
   <si>
     <t>Topic</t>
   </si>
@@ -7184,6 +7184,12 @@
   </si>
   <si>
     <t>menyatakan informasi belum menjadi bencana nasional dan menyatakan kritik</t>
+  </si>
+  <si>
+    <t>hanya menunjukkkan pandangan pemerintah</t>
+  </si>
+  <si>
+    <t>menyatakan dukungan terhadap penetapan bencana nasional</t>
   </si>
 </sst>
 </file>
@@ -8252,11 +8258,17 @@
         <v>8</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
+        <v>43</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>2188</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="O12" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="P12" s="3" t="s">
         <v>12</v>
       </c>
@@ -9548,7 +9560,9 @@
       <c r="L38" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M38" s="3"/>
+      <c r="M38" s="3" t="s">
+        <v>2182</v>
+      </c>
       <c r="N38" s="9" t="s">
         <v>45</v>
       </c>
@@ -10046,7 +10060,9 @@
       <c r="L48" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M48" s="3"/>
+      <c r="M48" s="3" t="s">
+        <v>2189</v>
+      </c>
       <c r="N48" s="9" t="s">
         <v>45</v>
       </c>
@@ -10194,7 +10210,9 @@
       <c r="L51" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="M51" s="3"/>
+      <c r="M51" s="3" t="s">
+        <v>2189</v>
+      </c>
       <c r="N51" s="9" t="s">
         <v>45</v>
       </c>
@@ -11898,7 +11916,9 @@
       <c r="N85" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="O85" s="3"/>
+      <c r="O85" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="P85" s="3" t="s">
         <v>12</v>
       </c>
@@ -11946,7 +11966,9 @@
       <c r="N86" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="O86" s="3"/>
+      <c r="O86" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="P86" s="3" t="s">
         <v>12</v>
       </c>
@@ -11994,7 +12016,9 @@
       <c r="N87" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="O87" s="3"/>
+      <c r="O87" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="P87" s="3" t="s">
         <v>12</v>
       </c>
@@ -13136,9 +13160,7 @@
       </c>
       <c r="M110" s="3"/>
       <c r="N110" s="3"/>
-      <c r="O110" s="2" t="s">
-        <v>46</v>
-      </c>
+      <c r="O110" s="9"/>
       <c r="P110" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
Labeling Part17 Final Labeling Audit and Model Handoff
</commit_message>
<xml_diff>
--- a/03_Labeling/outputs/full_annotation/full_annotation_381.xlsx
+++ b/03_Labeling/outputs/full_annotation/full_annotation_381.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Penelitian Sentimen Bencana Nasional\03_Labeling\outputs\full_annotation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A9B290-41C0-4EE3-A833-3A941ADDFEA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4066B7B-E111-4FFC-8F32-F1F957C8D4B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7874,7 +7874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>47</v>
       </c>
@@ -9174,7 +9174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="72" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>167</v>
       </c>
@@ -9424,7 +9424,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>47</v>
       </c>
@@ -9524,7 +9524,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>47</v>
       </c>
@@ -11174,7 +11174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>34</v>
       </c>
@@ -13924,7 +13924,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="125" spans="1:16" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
         <v>167</v>
       </c>
@@ -14074,7 +14074,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="128" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
         <v>167</v>
       </c>
@@ -14174,7 +14174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="1:16" ht="72" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
         <v>167</v>
       </c>
@@ -22174,7 +22174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="290" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A290" s="2" t="s">
         <v>47</v>
       </c>
@@ -25974,7 +25974,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="366" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A366" s="2" t="s">
         <v>167</v>
       </c>

</xml_diff>